<commit_message>
Streamlined efficiency parameters, improved performance
</commit_message>
<xml_diff>
--- a/gmx/Example_output_files/PSD_Plot.xlsx
+++ b/gmx/Example_output_files/PSD_Plot.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/42c400a6d2268350/Penn/GitHub/PrO-VAT/gmx/Example_output_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7149973D-7FBA-47E4-9186-8284705DD2B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="8_{7149973D-7FBA-47E4-9186-8284705DD2B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AC3E1AAB-673D-43C5-AFEF-5531247DDE1C}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D12CB501-9D5F-4141-A117-3B2D7216ADD7}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D12CB501-9D5F-4141-A117-3B2D7216ADD7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -3008,6 +3008,7 @@
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="642880847"/>
+        <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:spPr>

</xml_diff>

<commit_message>
Significantly improved readability of PrO-VAT.py
</commit_message>
<xml_diff>
--- a/gmx/Example_output_files/PSD_Plot.xlsx
+++ b/gmx/Example_output_files/PSD_Plot.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/42c400a6d2268350/Penn/GitHub/PrO-VAT/gmx/Example_output_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="19" documentId="8_{7149973D-7FBA-47E4-9186-8284705DD2B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{23F376C0-B913-49C2-8D20-648CE629DA60}"/>
+  <xr:revisionPtr revIDLastSave="51" documentId="8_{7149973D-7FBA-47E4-9186-8284705DD2B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{35EC965B-3678-404F-9067-CA485303A5A5}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D12CB501-9D5F-4141-A117-3B2D7216ADD7}"/>
   </bookViews>
@@ -3479,7 +3479,7 @@
         <v>19.149999999999999</v>
       </c>
       <c r="B67">
-        <f t="shared" ref="B67:B130" si="1">A67/10</f>
+        <f t="shared" ref="B67:B74" si="1">A67/10</f>
         <v>1.9149999999999998</v>
       </c>
       <c r="C67">

</xml_diff>